<commit_message>
feature/fsel-4793: Update Code Get File Report
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/Report_School_Student.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/Report_School_Student.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PhanPhuc\Fsel\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF272D1A-F88D-499F-96D3-B832435D7182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14CEA3F6-D33B-4E8B-A754-C1885E488E1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CDA82A5-A310-4641-B205-387C49AE4D30}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>STT</t>
   </si>
@@ -76,6 +76,24 @@
   </si>
   <si>
     <t>Số bình luận trên bài đăng</t>
+  </si>
+  <si>
+    <t>Trường</t>
+  </si>
+  <si>
+    <t>Khối</t>
+  </si>
+  <si>
+    <t>LocalId</t>
+  </si>
+  <si>
+    <t>GlobalId</t>
+  </si>
+  <si>
+    <t>EventCode</t>
+  </si>
+  <si>
+    <t>UserName</t>
   </si>
 </sst>
 </file>
@@ -157,7 +175,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -254,13 +272,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -273,6 +300,12 @@
     </xf>
     <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -629,113 +662,152 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CE3A801-9DA4-4B8C-A876-F4C15216E3C6}">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="21" max="21" width="9.875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:21" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="I1" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="11" t="s">
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="13" t="s">
         <v>6</v>
       </c>
+      <c r="S1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="T1" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="U1" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="9"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="13" t="s">
+    <row r="2" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="14"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="13" t="s">
+      <c r="J2" s="16"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="16" t="s">
+      <c r="M2" s="17"/>
+      <c r="N2" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="17"/>
-      <c r="M2" s="13" t="s">
+      <c r="O2" s="19"/>
+      <c r="P2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="N2" s="15"/>
-      <c r="O2" s="11"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="5"/>
+      <c r="T2" s="6"/>
+      <c r="U2" s="6"/>
     </row>
-    <row r="3" spans="1:15" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A3" s="10"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="1" t="s">
+    <row r="3" spans="1:21" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="M3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="N3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="P3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O3" s="11"/>
+      <c r="R3" s="13"/>
+      <c r="S3" s="5"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="D1:D3"/>
-    <mergeCell ref="C1:C3"/>
+  <mergeCells count="17">
     <mergeCell ref="B1:B3"/>
     <mergeCell ref="A1:A3"/>
-    <mergeCell ref="O1:O3"/>
-    <mergeCell ref="F1:N1"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="R1:R3"/>
+    <mergeCell ref="I1:Q1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="H1:H3"/>
+    <mergeCell ref="F1:F3"/>
+    <mergeCell ref="G1:G3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="S1:S3"/>
+    <mergeCell ref="T1:T3"/>
+    <mergeCell ref="U1:U3"/>
     <mergeCell ref="E1:E3"/>
+    <mergeCell ref="D1:D3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feature/fsel-6095: Update Fix Report
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/Report_School_Student.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/Report_School_Student.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PhanPhuc\Fsel\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14CEA3F6-D33B-4E8B-A754-C1885E488E1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB3B0B02-B5EB-4E16-97B4-B4B2CE2520CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CDA82A5-A310-4641-B205-387C49AE4D30}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>STT</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Tiêu chí đánh giá Tuần 1</t>
   </si>
   <si>
-    <t>Tổng điểm</t>
-  </si>
-  <si>
     <t>Tiến trình tự học</t>
   </si>
   <si>
@@ -94,6 +91,15 @@
   </si>
   <si>
     <t>UserName</t>
+  </si>
+  <si>
+    <t>Tổng điểm theo công thức hà nội</t>
+  </si>
+  <si>
+    <t>ContentComplete</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tổng điểm tháng tự học </t>
   </si>
 </sst>
 </file>
@@ -164,18 +170,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -272,22 +278,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -301,49 +298,56 @@
     <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="5" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="5" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -662,138 +666,156 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CE3A801-9DA4-4B8C-A876-F4C15216E3C6}">
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:W3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="21" max="21" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="9" style="18"/>
+    <col min="23" max="23" width="9.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:23" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="G1" s="7" t="s">
+      <c r="S1" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="T1" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="U1" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="H1" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
-      <c r="P1" s="14"/>
-      <c r="Q1" s="14"/>
-      <c r="R1" s="13" t="s">
+      <c r="V1" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="W1" s="19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="S1" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="T1" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="U1" s="6" t="s">
-        <v>21</v>
-      </c>
+      <c r="J2" s="10"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="11"/>
+      <c r="N2" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="O2" s="13"/>
+      <c r="P2" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="17"/>
+      <c r="S2" s="21"/>
+      <c r="T2" s="21"/>
+      <c r="U2" s="19"/>
+      <c r="V2" s="19"/>
+      <c r="W2" s="19"/>
     </row>
-    <row r="2" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="J2" s="16"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="M2" s="17"/>
-      <c r="N2" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="O2" s="19"/>
-      <c r="P2" s="15" t="s">
+    <row r="3" spans="1:23" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="17"/>
-      <c r="R2" s="13"/>
-      <c r="S2" s="5"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="6"/>
-    </row>
-    <row r="3" spans="1:21" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="M3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="M3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="N3" s="3" t="s">
+      <c r="O3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="O3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="Q3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="R3" s="13"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
+        <v>12</v>
+      </c>
+      <c r="R3" s="17"/>
+      <c r="S3" s="22"/>
+      <c r="T3" s="22"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+      <c r="W3" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="19">
+    <mergeCell ref="U1:U3"/>
+    <mergeCell ref="V1:V3"/>
+    <mergeCell ref="W1:W3"/>
+    <mergeCell ref="E1:E3"/>
+    <mergeCell ref="D1:D3"/>
+    <mergeCell ref="R1:R3"/>
+    <mergeCell ref="S1:S3"/>
+    <mergeCell ref="T1:T3"/>
     <mergeCell ref="B1:B3"/>
     <mergeCell ref="A1:A3"/>
-    <mergeCell ref="R1:R3"/>
     <mergeCell ref="I1:Q1"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="L2:M2"/>
@@ -803,11 +825,6 @@
     <mergeCell ref="F1:F3"/>
     <mergeCell ref="G1:G3"/>
     <mergeCell ref="C1:C3"/>
-    <mergeCell ref="S1:S3"/>
-    <mergeCell ref="T1:T3"/>
-    <mergeCell ref="U1:U3"/>
-    <mergeCell ref="E1:E3"/>
-    <mergeCell ref="D1:D3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feature/fsel-6095: Update Export File Student
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/Report_School_Student.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/Report_School_Student.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB3B0B02-B5EB-4E16-97B4-B4B2CE2520CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8979DCB1-F847-47C7-8DB2-72752ADBF8F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CDA82A5-A310-4641-B205-387C49AE4D30}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
     <t>STT</t>
   </si>
@@ -96,10 +96,13 @@
     <t>Tổng điểm theo công thức hà nội</t>
   </si>
   <si>
-    <t>ContentComplete</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tổng điểm tháng tự học </t>
+  </si>
+  <si>
+    <t>Nội dung dã hoàn thành</t>
+  </si>
+  <si>
+    <t>Tổng số nội dung</t>
   </si>
 </sst>
 </file>
@@ -284,7 +287,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -298,6 +301,18 @@
     <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -307,6 +322,9 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -323,31 +341,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -666,110 +659,113 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CE3A801-9DA4-4B8C-A876-F4C15216E3C6}">
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:X3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="19" max="20" width="9" style="18"/>
-    <col min="23" max="23" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:24" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="17" t="s">
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="S1" s="20" t="s">
+      <c r="S1" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="T1" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="T1" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="U1" s="19" t="s">
+      <c r="V1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="V1" s="19" t="s">
+      <c r="W1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="W1" s="19" t="s">
+      <c r="X1" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="9" t="s">
+    <row r="2" spans="1:24" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="10"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="10"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="9" t="s">
+      <c r="J2" s="15"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="11"/>
-      <c r="N2" s="12" t="s">
+      <c r="M2" s="16"/>
+      <c r="N2" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="13"/>
-      <c r="P2" s="9" t="s">
+      <c r="O2" s="18"/>
+      <c r="P2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="17"/>
-      <c r="S2" s="21"/>
-      <c r="T2" s="21"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="19"/>
-      <c r="W2" s="19"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
+      <c r="V2" s="5"/>
+      <c r="W2" s="5"/>
+      <c r="X2" s="5"/>
     </row>
-    <row r="3" spans="1:23" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
+    <row r="3" spans="1:24" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A3" s="11"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
       <c r="I3" s="1" t="s">
         <v>10</v>
       </c>
@@ -797,23 +793,16 @@
       <c r="Q3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="17"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="19"/>
-      <c r="V3" s="19"/>
-      <c r="W3" s="19"/>
+      <c r="R3" s="12"/>
+      <c r="S3" s="12"/>
+      <c r="T3" s="12"/>
+      <c r="U3" s="12"/>
+      <c r="V3" s="5"/>
+      <c r="W3" s="5"/>
+      <c r="X3" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="U1:U3"/>
-    <mergeCell ref="V1:V3"/>
-    <mergeCell ref="W1:W3"/>
-    <mergeCell ref="E1:E3"/>
-    <mergeCell ref="D1:D3"/>
-    <mergeCell ref="R1:R3"/>
-    <mergeCell ref="S1:S3"/>
-    <mergeCell ref="T1:T3"/>
+  <mergeCells count="20">
     <mergeCell ref="B1:B3"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="I1:Q1"/>
@@ -825,6 +814,15 @@
     <mergeCell ref="F1:F3"/>
     <mergeCell ref="G1:G3"/>
     <mergeCell ref="C1:C3"/>
+    <mergeCell ref="V1:V3"/>
+    <mergeCell ref="W1:W3"/>
+    <mergeCell ref="X1:X3"/>
+    <mergeCell ref="E1:E3"/>
+    <mergeCell ref="D1:D3"/>
+    <mergeCell ref="R1:R3"/>
+    <mergeCell ref="S1:S3"/>
+    <mergeCell ref="U1:U3"/>
+    <mergeCell ref="T1:T3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
FSEL-8537: fix report student by event
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/Report_School_Student.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/Report_School_Student.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\multiple-subject\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8979DCB1-F847-47C7-8DB2-72752ADBF8F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CDA82A5-A310-4641-B205-387C49AE4D30}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="152511" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>STT</t>
   </si>
@@ -60,18 +59,9 @@
     <t>Số lượng hoàn thành bài học</t>
   </si>
   <si>
-    <t>Tỷ lệ hoàn thành chỉ tiêu</t>
-  </si>
-  <si>
-    <t>Mức điểm</t>
-  </si>
-  <si>
     <t>Điểm đạt được</t>
   </si>
   <si>
-    <t>Tỷ lệ hoàn thành bài tập</t>
-  </si>
-  <si>
     <t>Số bình luận trên bài đăng</t>
   </si>
   <si>
@@ -93,40 +83,37 @@
     <t>UserName</t>
   </si>
   <si>
-    <t>Tổng điểm theo công thức hà nội</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tổng điểm tháng tự học </t>
-  </si>
-  <si>
     <t>Nội dung dã hoàn thành</t>
   </si>
   <si>
     <t>Tổng số nội dung</t>
+  </si>
+  <si>
+    <t>Số lượng bài Classforum đã hoàn thành</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -184,7 +171,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -221,30 +208,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -287,7 +250,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -295,59 +258,50 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{79933E24-1CB4-4146-AA0D-6A00E0457A8C}"/>
-    <cellStyle name="Percent 2" xfId="2" xr:uid="{A81696F5-ABCE-42F2-A023-27911B028FC5}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Percent 2" xfId="2"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -658,171 +612,130 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CE3A801-9DA4-4B8C-A876-F4C15216E3C6}">
-  <dimension ref="A1:X3"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Q3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="24" max="24" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" s="9" t="s">
+      <c r="C1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="N1" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="P1" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="Q1" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13"/>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13"/>
-      <c r="R1" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="S1" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="T1" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="U1" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="V1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="W1" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="X1" s="5" t="s">
-        <v>20</v>
-      </c>
     </row>
-    <row r="2" spans="1:24" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="14" t="s">
+    <row r="2" spans="1:17" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="14" t="s">
+      <c r="J2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="16"/>
-      <c r="N2" s="17" t="s">
+      <c r="K2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="18"/>
-      <c r="P2" s="14" t="s">
+      <c r="L2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
-      <c r="U2" s="12"/>
-      <c r="V2" s="5"/>
-      <c r="W2" s="5"/>
-      <c r="X2" s="5"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
     </row>
-    <row r="3" spans="1:24" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
+    <row r="3" spans="1:17" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
       <c r="I3" s="1" t="s">
         <v>10</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-      <c r="T3" s="12"/>
-      <c r="U3" s="12"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="5"/>
-      <c r="X3" s="5"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="14">
+    <mergeCell ref="O1:O3"/>
+    <mergeCell ref="P1:P3"/>
+    <mergeCell ref="Q1:Q3"/>
+    <mergeCell ref="E1:E3"/>
+    <mergeCell ref="D1:D3"/>
+    <mergeCell ref="M1:M3"/>
+    <mergeCell ref="N1:N3"/>
     <mergeCell ref="B1:B3"/>
     <mergeCell ref="A1:A3"/>
-    <mergeCell ref="I1:Q1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="I1:L1"/>
     <mergeCell ref="H1:H3"/>
     <mergeCell ref="F1:F3"/>
     <mergeCell ref="G1:G3"/>
     <mergeCell ref="C1:C3"/>
-    <mergeCell ref="V1:V3"/>
-    <mergeCell ref="W1:W3"/>
-    <mergeCell ref="X1:X3"/>
-    <mergeCell ref="E1:E3"/>
-    <mergeCell ref="D1:D3"/>
-    <mergeCell ref="R1:R3"/>
-    <mergeCell ref="S1:S3"/>
-    <mergeCell ref="U1:U3"/>
-    <mergeCell ref="T1:T3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>